<commit_message>
added main.py into app folder
</commit_message>
<xml_diff>
--- a/baza/Kostka Lagerplatz.xlsx
+++ b/baza/Kostka Lagerplatz.xlsx
@@ -3567,7 +3567,7 @@
         </is>
       </c>
       <c r="D173" s="3" t="n">
-        <v>167</v>
+        <v>227</v>
       </c>
     </row>
     <row r="174" ht="17.25" customHeight="1">
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="D174" s="3" t="n">
-        <v>167</v>
+        <v>227</v>
       </c>
     </row>
     <row r="175" ht="17.25" customHeight="1">
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="D175" s="3" t="n">
-        <v>166</v>
+        <v>226</v>
       </c>
     </row>
     <row r="176" ht="17.25" customHeight="1">
@@ -3621,7 +3621,7 @@
         </is>
       </c>
       <c r="D176" s="3" t="n">
-        <v>167</v>
+        <v>227</v>
       </c>
     </row>
     <row r="177" ht="17.25" customHeight="1">
@@ -3819,7 +3819,7 @@
         </is>
       </c>
       <c r="D187" s="3" t="n">
-        <v>167</v>
+        <v>227</v>
       </c>
     </row>
     <row r="188" ht="17.25" customHeight="1">
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="D188" s="3" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
     </row>
     <row r="189" ht="17.25" customHeight="1">
@@ -3855,7 +3855,7 @@
         </is>
       </c>
       <c r="D189" s="3" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
     </row>
     <row r="190" ht="17.25" customHeight="1">
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="D246" s="3" t="n">
-        <v>41</v>
+        <v>56</v>
       </c>
     </row>
     <row r="247" ht="17.25" customHeight="1">
@@ -5169,7 +5169,7 @@
         </is>
       </c>
       <c r="D262" s="3" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="263" ht="17.25" customHeight="1">

</xml_diff>

<commit_message>
added clean log and git ignroe
</commit_message>
<xml_diff>
--- a/baza/Kostka Lagerplatz.xlsx
+++ b/baza/Kostka Lagerplatz.xlsx
@@ -3567,7 +3567,7 @@
         </is>
       </c>
       <c r="D173" s="3" t="n">
-        <v>227</v>
+        <v>267</v>
       </c>
     </row>
     <row r="174" ht="17.25" customHeight="1">
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="D174" s="3" t="n">
-        <v>227</v>
+        <v>267</v>
       </c>
     </row>
     <row r="175" ht="17.25" customHeight="1">
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="D175" s="3" t="n">
-        <v>226</v>
+        <v>266</v>
       </c>
     </row>
     <row r="176" ht="17.25" customHeight="1">
@@ -3621,7 +3621,7 @@
         </is>
       </c>
       <c r="D176" s="3" t="n">
-        <v>227</v>
+        <v>267</v>
       </c>
     </row>
     <row r="177" ht="17.25" customHeight="1">
@@ -3819,7 +3819,7 @@
         </is>
       </c>
       <c r="D187" s="3" t="n">
-        <v>227</v>
+        <v>267</v>
       </c>
     </row>
     <row r="188" ht="17.25" customHeight="1">
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="D188" s="3" t="n">
-        <v>180</v>
+        <v>220</v>
       </c>
     </row>
     <row r="189" ht="17.25" customHeight="1">
@@ -3855,7 +3855,7 @@
         </is>
       </c>
       <c r="D189" s="3" t="n">
-        <v>180</v>
+        <v>220</v>
       </c>
     </row>
     <row r="190" ht="17.25" customHeight="1">
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="D246" s="3" t="n">
-        <v>56</v>
+        <v>66</v>
       </c>
     </row>
     <row r="247" ht="17.25" customHeight="1">
@@ -5169,7 +5169,7 @@
         </is>
       </c>
       <c r="D262" s="3" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="263" ht="17.25" customHeight="1">

</xml_diff>